<commit_message>
feat(plan): jalons des objectifs clés tirés du classeur
À l'import, chaque objectif clé reçoit des jalons datés jusqu'à son
échéance : la trajectoire de l'enveloppe qu'il vise (par son nom ou le
montant de sa cible) et les lignes du journal ou primes qui en parlent
(un mot rare en commun, ou deux mots ; lieux et mots courants écartés).
Un réimport en ajoute aux objectifs déjà là qui n'en ont aucun ; un
objectif atteint a ses jalons cochés. Aucun jalon plutôt qu'un jalon
hors sujet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012LFZsBkWXSQjKa1Kmywgod
</commit_message>
<xml_diff>
--- a/src/features/plan/__fixtures__/plan-fictif.xlsx
+++ b/src/features/plan/__fixtures__/plan-fictif.xlsx
@@ -1754,6 +1754,18 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Déc 2028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Déposer la demande de résidence permanente</t>
+        </is>
+      </c>
+    </row>
     <row r="200">
       <c r="A200">
         <f>C35</f>

</xml_diff>